<commit_message>
I thought these were already commited?
</commit_message>
<xml_diff>
--- a/144/DQ Templates and Instructions/Topic 1 DQ 1/Topic 1 DQ 1.xlsx
+++ b/144/DQ Templates and Instructions/Topic 1 DQ 1/Topic 1 DQ 1.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gcumail.sharepoint.com/sites/MathematicsProgramFacultyStaff-MATOFTF/Shared Documents/MATOFTF/ALEKS/DQ Templates and Instructions/Topic 1 DQ 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="124" documentId="8_{197DFB2F-3D6E-4006-9337-6C654C7D47B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{351851BE-7648-408A-95BF-C14B0DF02E34}"/>
+  <xr:revisionPtr revIDLastSave="172" documentId="8_{197DFB2F-3D6E-4006-9337-6C654C7D47B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06D602D3-C1FE-44AC-B081-604E055F858C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4FCF7FA6-22BB-4545-AB27-D5B8AACA448D}"/>
   </bookViews>
   <sheets>
     <sheet name="Goals and Instructions" sheetId="4" r:id="rId1"/>
     <sheet name="Basic Excel Formulas" sheetId="1" r:id="rId2"/>
-    <sheet name="Solutions" sheetId="2" state="hidden" r:id="rId3"/>
-    <sheet name="Sheet2" sheetId="3" state="hidden" r:id="rId4"/>
+    <sheet name="Users" sheetId="5" state="hidden" r:id="rId3"/>
+    <sheet name="Solutions" sheetId="2" state="hidden" r:id="rId4"/>
+    <sheet name="Sheet2" sheetId="3" state="hidden" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="CHECKDIV">_xlfn.LAMBDA(_xlpm.x,AND(_xlpm.x &lt;&gt; "", IFERROR(AND(     SUBSTITUTE(_xlfn.FORMULATEXT(_xlpm.x), " ","") &lt;&gt; "=B8/C8",  SUBSTITUTE(_xlfn.FORMULATEXT(_xlpm.x), " ","") &lt;&gt; "=SUM(B8/C8)",  SUBSTITUTE(_xlfn.FORMULATEXT(_xlpm.x), " ","") &lt;&gt; "=(B8/C8)"), TRUE)))</definedName>
@@ -27,7 +28,7 @@
     <definedName name="CHECKSUM">_xlfn.LAMBDA(_xlpm.x,AND(_xlpm.x &lt;&gt; "", IFERROR(AND(     SUBSTITUTE(_xlfn.FORMULATEXT(_xlpm.x), " ","") &lt;&gt; "=B8+C8",  SUBSTITUTE(_xlfn.FORMULATEXT(_xlpm.x), " ","") &lt;&gt; "=C8+B8",  SUBSTITUTE(_xlfn.FORMULATEXT(_xlpm.x), " ","") &lt;&gt; "=SUM(C8,B8)",  SUBSTITUTE(_xlfn.FORMULATEXT(_xlpm.x), " ","") &lt;&gt; "=SUM(B8,C8)",  SUBSTITUTE(_xlfn.FORMULATEXT(_xlpm.x), " ","") &lt;&gt; "=(C8+B8)",  SUBSTITUTE(_xlfn.FORMULATEXT(_xlpm.x), " ","") &lt;&gt; "=(B8+C8)"), TRUE)))</definedName>
     <definedName name="checksys">_xlfn.LAMBDA(IFERROR(IF(ISURL("http://g.co"), "Google Sheets"),IFERROR(IF(DUR2DAYS("1d")&gt;0, "Apple Numbers"),IF(ISERROR(INFO("directory")), "Excel Online", "Excel Desktop"))))</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -97,7 +98,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="84">
   <si>
     <t>Excel skills to be learned</t>
   </si>
@@ -461,6 +462,12 @@
   <si>
     <t>Your Name Here</t>
   </si>
+  <si>
+    <t>Names</t>
+  </si>
+  <si>
+    <t>Reset</t>
+  </si>
 </sst>
 </file>
 
@@ -469,7 +476,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode=";;;"/>
   </numFmts>
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -595,12 +602,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -1225,7 +1226,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="192">
+  <cellXfs count="194">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1355,22 +1356,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="26" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
@@ -1519,6 +1520,134 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1593,133 +1722,47 @@
       <alignment horizontal="left" indent="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="21" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="32" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1747,24 +1790,6 @@
     <xf numFmtId="0" fontId="9" fillId="12" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1" indent="1"/>
     </xf>
@@ -1774,30 +1799,6 @@
     <xf numFmtId="0" fontId="9" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="12" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1824,6 +1825,13 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2528,94 +2536,94 @@
       <c r="A1" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="L1" s="107" t="str">
+      <c r="L1" s="147" t="str">
         <f ca="1">IF(OR(I2="Excel Desktop",I2="Excel Online"),"","You are not using Excel, please proceed to office.com, log in with your GCU credentials, and install the current Office 365, or use the online versions. Work not completed in Excel must be redone.")</f>
         <v/>
       </c>
-      <c r="M1" s="108"/>
-      <c r="N1" s="108"/>
-      <c r="O1" s="109"/>
+      <c r="M1" s="148"/>
+      <c r="N1" s="148"/>
+      <c r="O1" s="149"/>
     </row>
     <row r="2" spans="1:15" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B2" s="31"/>
-      <c r="C2" s="101" t="s">
+      <c r="C2" s="141" t="s">
         <v>13</v>
       </c>
-      <c r="D2" s="102"/>
-      <c r="E2" s="103"/>
+      <c r="D2" s="142"/>
+      <c r="E2" s="143"/>
       <c r="G2" s="29" t="s">
         <v>14</v>
       </c>
       <c r="H2" s="32" t="s">
         <v>81</v>
       </c>
-      <c r="I2" s="99" t="str" cm="1">
+      <c r="I2" s="139" t="str" cm="1">
         <f t="array" aca="1" ref="I2" ca="1">checksys()</f>
         <v>Excel Desktop</v>
       </c>
-      <c r="J2" s="100"/>
-      <c r="L2" s="110"/>
-      <c r="M2" s="111"/>
-      <c r="N2" s="111"/>
-      <c r="O2" s="112"/>
+      <c r="J2" s="140"/>
+      <c r="L2" s="150"/>
+      <c r="M2" s="151"/>
+      <c r="N2" s="151"/>
+      <c r="O2" s="152"/>
     </row>
     <row r="3" spans="1:15" ht="23.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="31"/>
-      <c r="C3" s="101" t="s">
+      <c r="C3" s="141" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="102"/>
-      <c r="E3" s="103"/>
-      <c r="L3" s="113"/>
-      <c r="M3" s="114"/>
-      <c r="N3" s="114"/>
-      <c r="O3" s="115"/>
+      <c r="D3" s="142"/>
+      <c r="E3" s="143"/>
+      <c r="L3" s="153"/>
+      <c r="M3" s="154"/>
+      <c r="N3" s="154"/>
+      <c r="O3" s="155"/>
     </row>
     <row r="4" spans="1:15" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="120" t="s">
+      <c r="B4" s="94" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="121"/>
-      <c r="D4" s="121"/>
-      <c r="E4" s="121"/>
-      <c r="F4" s="122"/>
-      <c r="M4" s="96" t="s">
+      <c r="C4" s="95"/>
+      <c r="D4" s="95"/>
+      <c r="E4" s="95"/>
+      <c r="F4" s="96"/>
+      <c r="M4" s="136" t="s">
         <v>10</v>
       </c>
-      <c r="N4" s="97"/>
+      <c r="N4" s="137"/>
     </row>
     <row r="5" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="123"/>
-      <c r="C5" s="124"/>
-      <c r="D5" s="124"/>
-      <c r="E5" s="124"/>
-      <c r="F5" s="125"/>
-      <c r="M5" s="98" t="s">
+      <c r="B5" s="97"/>
+      <c r="C5" s="98"/>
+      <c r="D5" s="98"/>
+      <c r="E5" s="98"/>
+      <c r="F5" s="99"/>
+      <c r="M5" s="138" t="s">
         <v>11</v>
       </c>
-      <c r="N5" s="98"/>
+      <c r="N5" s="138"/>
     </row>
     <row r="6" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B6" s="126" t="s">
+      <c r="B6" s="122" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="127"/>
-      <c r="D6" s="149" t="s">
+      <c r="C6" s="123"/>
+      <c r="D6" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="151" t="s">
+      <c r="E6" s="105" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="136" t="s">
+      <c r="F6" s="132" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="156" t="s">
+      <c r="G6" s="110" t="s">
         <v>21</v>
       </c>
-      <c r="I6" s="128" t="s">
+      <c r="I6" s="124" t="s">
         <v>22</v>
       </c>
-      <c r="J6" s="129"/>
+      <c r="J6" s="125"/>
     </row>
     <row r="7" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
@@ -2624,10 +2632,10 @@
       <c r="C7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="150"/>
-      <c r="E7" s="152"/>
-      <c r="F7" s="137"/>
-      <c r="G7" s="157"/>
+      <c r="D7" s="104"/>
+      <c r="E7" s="106"/>
+      <c r="F7" s="133"/>
+      <c r="G7" s="111"/>
       <c r="I7" s="18" t="s">
         <v>25</v>
       </c>
@@ -2656,10 +2664,10 @@
       </c>
     </row>
     <row r="9" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B9" s="130" t="s">
+      <c r="B9" s="126" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="131"/>
+      <c r="C9" s="127"/>
       <c r="D9" s="2" t="s">
         <v>33</v>
       </c>
@@ -2678,8 +2686,8 @@
       </c>
     </row>
     <row r="10" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B10" s="132"/>
-      <c r="C10" s="133"/>
+      <c r="B10" s="128"/>
+      <c r="C10" s="129"/>
       <c r="D10" s="2" t="s">
         <v>38</v>
       </c>
@@ -2698,8 +2706,8 @@
       </c>
     </row>
     <row r="11" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="132"/>
-      <c r="C11" s="133"/>
+      <c r="B11" s="128"/>
+      <c r="C11" s="129"/>
       <c r="D11" s="2" t="s">
         <v>43</v>
       </c>
@@ -2718,8 +2726,8 @@
       </c>
     </row>
     <row r="12" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="134"/>
-      <c r="C12" s="135"/>
+      <c r="B12" s="130"/>
+      <c r="C12" s="131"/>
       <c r="D12" s="7" t="s">
         <v>48</v>
       </c>
@@ -2732,19 +2740,19 @@
       </c>
     </row>
     <row r="13" spans="1:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="153" t="s">
+      <c r="B13" s="107" t="s">
         <v>51</v>
       </c>
-      <c r="C13" s="154"/>
-      <c r="D13" s="154"/>
-      <c r="E13" s="154"/>
-      <c r="F13" s="155"/>
-      <c r="I13" s="104" t="s">
+      <c r="C13" s="108"/>
+      <c r="D13" s="108"/>
+      <c r="E13" s="108"/>
+      <c r="F13" s="109"/>
+      <c r="I13" s="144" t="s">
         <v>52</v>
       </c>
-      <c r="J13" s="105"/>
-      <c r="K13" s="105"/>
-      <c r="L13" s="106"/>
+      <c r="J13" s="145"/>
+      <c r="K13" s="145"/>
+      <c r="L13" s="146"/>
     </row>
     <row r="14" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="42"/>
@@ -2755,17 +2763,17 @@
       <c r="H14" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="I14" s="116" t="s">
+      <c r="I14" s="156" t="s">
         <v>54</v>
       </c>
-      <c r="J14" s="116"/>
-      <c r="K14" s="116"/>
-      <c r="L14" s="117"/>
-      <c r="M14" s="94" t="s">
+      <c r="J14" s="156"/>
+      <c r="K14" s="156"/>
+      <c r="L14" s="157"/>
+      <c r="M14" s="134" t="s">
         <v>55</v>
       </c>
-      <c r="N14" s="95"/>
-      <c r="O14" s="95"/>
+      <c r="N14" s="135"/>
+      <c r="O14" s="135"/>
     </row>
     <row r="15" spans="1:15" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="13"/>
@@ -2774,12 +2782,12 @@
       <c r="H15" s="35">
         <v>15</v>
       </c>
-      <c r="I15" s="118" t="s">
+      <c r="I15" s="120" t="s">
         <v>56</v>
       </c>
-      <c r="J15" s="118"/>
-      <c r="K15" s="118"/>
-      <c r="L15" s="119"/>
+      <c r="J15" s="120"/>
+      <c r="K15" s="120"/>
+      <c r="L15" s="121"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B16" s="13"/>
@@ -2788,47 +2796,47 @@
       <c r="H16" s="27">
         <v>16</v>
       </c>
-      <c r="I16" s="138" t="s">
+      <c r="I16" s="112" t="s">
         <v>57</v>
       </c>
-      <c r="J16" s="138"/>
-      <c r="K16" s="138"/>
-      <c r="L16" s="139"/>
+      <c r="J16" s="112"/>
+      <c r="K16" s="112"/>
+      <c r="L16" s="113"/>
     </row>
     <row r="17" spans="2:12" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="12"/>
       <c r="H17" s="28">
         <v>16</v>
       </c>
-      <c r="I17" s="140" t="s">
+      <c r="I17" s="114" t="s">
         <v>58</v>
       </c>
-      <c r="J17" s="140"/>
-      <c r="K17" s="140"/>
-      <c r="L17" s="141"/>
+      <c r="J17" s="114"/>
+      <c r="K17" s="114"/>
+      <c r="L17" s="115"/>
     </row>
     <row r="18" spans="2:12" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="120" t="s">
+      <c r="B18" s="94" t="s">
         <v>59</v>
       </c>
-      <c r="C18" s="121"/>
-      <c r="D18" s="121"/>
-      <c r="E18" s="121"/>
-      <c r="F18" s="122"/>
+      <c r="C18" s="95"/>
+      <c r="D18" s="95"/>
+      <c r="E18" s="95"/>
+      <c r="F18" s="96"/>
     </row>
     <row r="19" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="123"/>
-      <c r="C19" s="124"/>
-      <c r="D19" s="124"/>
-      <c r="E19" s="124"/>
-      <c r="F19" s="125"/>
+      <c r="B19" s="97"/>
+      <c r="C19" s="98"/>
+      <c r="D19" s="98"/>
+      <c r="E19" s="98"/>
+      <c r="F19" s="99"/>
     </row>
     <row r="20" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="146" t="s">
+      <c r="B20" s="100" t="s">
         <v>80</v>
       </c>
-      <c r="C20" s="146"/>
-      <c r="D20" s="146"/>
+      <c r="C20" s="100"/>
+      <c r="D20" s="100"/>
       <c r="E20" s="10" t="s">
         <v>60</v>
       </c>
@@ -2839,15 +2847,15 @@
         <v>62</v>
       </c>
       <c r="H20" s="17"/>
-      <c r="I20" s="144" t="s">
+      <c r="I20" s="118" t="s">
         <v>63</v>
       </c>
-      <c r="J20" s="145"/>
+      <c r="J20" s="119"/>
     </row>
     <row r="21" spans="2:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B21" s="147"/>
-      <c r="C21" s="147"/>
-      <c r="D21" s="147"/>
+      <c r="B21" s="101"/>
+      <c r="C21" s="101"/>
+      <c r="D21" s="101"/>
       <c r="E21" s="33"/>
       <c r="F21" s="2" t="s">
         <v>64</v>
@@ -2856,15 +2864,15 @@
         <v>65</v>
       </c>
       <c r="H21" s="41"/>
-      <c r="I21" s="142" t="s">
+      <c r="I21" s="116" t="s">
         <v>66</v>
       </c>
-      <c r="J21" s="142"/>
+      <c r="J21" s="116"/>
     </row>
     <row r="22" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B22" s="147"/>
-      <c r="C22" s="147"/>
-      <c r="D22" s="147"/>
+      <c r="B22" s="101"/>
+      <c r="C22" s="101"/>
+      <c r="D22" s="101"/>
       <c r="E22" s="33"/>
       <c r="F22" s="2" t="s">
         <v>67</v>
@@ -2873,15 +2881,15 @@
         <v>68</v>
       </c>
       <c r="H22" s="41"/>
-      <c r="I22" s="143" t="s">
+      <c r="I22" s="117" t="s">
         <v>69</v>
       </c>
-      <c r="J22" s="143"/>
+      <c r="J22" s="117"/>
     </row>
     <row r="23" spans="2:12" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B23" s="147"/>
-      <c r="C23" s="147"/>
-      <c r="D23" s="147"/>
+      <c r="B23" s="101"/>
+      <c r="C23" s="101"/>
+      <c r="D23" s="101"/>
       <c r="E23" s="33"/>
       <c r="F23" s="2" t="s">
         <v>70</v>
@@ -2890,64 +2898,64 @@
         <v>71</v>
       </c>
       <c r="H23" s="41"/>
-      <c r="I23" s="143" t="s">
+      <c r="I23" s="117" t="s">
         <v>72</v>
       </c>
-      <c r="J23" s="143"/>
+      <c r="J23" s="117"/>
     </row>
     <row r="24" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B24" s="147"/>
-      <c r="C24" s="147"/>
-      <c r="D24" s="147"/>
+      <c r="B24" s="101"/>
+      <c r="C24" s="101"/>
+      <c r="D24" s="101"/>
       <c r="E24" s="33"/>
-      <c r="F24" s="148" t="s">
+      <c r="F24" s="102" t="s">
         <v>73</v>
       </c>
-      <c r="G24" s="148"/>
+      <c r="G24" s="102"/>
       <c r="H24" s="36"/>
       <c r="I24" s="37"/>
       <c r="J24" s="37"/>
     </row>
     <row r="25" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B25" s="147"/>
-      <c r="C25" s="147"/>
-      <c r="D25" s="147"/>
+      <c r="B25" s="101"/>
+      <c r="C25" s="101"/>
+      <c r="D25" s="101"/>
       <c r="E25" s="33"/>
-      <c r="F25" s="148"/>
-      <c r="G25" s="148"/>
+      <c r="F25" s="102"/>
+      <c r="G25" s="102"/>
       <c r="H25" s="38"/>
       <c r="I25" s="39"/>
       <c r="J25" s="39"/>
     </row>
     <row r="26" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B26" s="147"/>
-      <c r="C26" s="147"/>
-      <c r="D26" s="147"/>
+      <c r="B26" s="101"/>
+      <c r="C26" s="101"/>
+      <c r="D26" s="101"/>
       <c r="E26" s="33"/>
-      <c r="F26" s="148"/>
-      <c r="G26" s="148"/>
+      <c r="F26" s="102"/>
+      <c r="G26" s="102"/>
       <c r="H26" s="38"/>
       <c r="I26" s="39"/>
       <c r="J26" s="39"/>
     </row>
     <row r="27" spans="2:12" x14ac:dyDescent="0.25">
-      <c r="B27" s="147"/>
-      <c r="C27" s="147"/>
-      <c r="D27" s="147"/>
+      <c r="B27" s="101"/>
+      <c r="C27" s="101"/>
+      <c r="D27" s="101"/>
       <c r="E27" s="33"/>
-      <c r="F27" s="148"/>
-      <c r="G27" s="148"/>
+      <c r="F27" s="102"/>
+      <c r="G27" s="102"/>
       <c r="H27" s="38"/>
       <c r="I27" s="39"/>
       <c r="J27" s="39"/>
     </row>
     <row r="28" spans="2:12" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="147"/>
-      <c r="C28" s="147"/>
-      <c r="D28" s="147"/>
+      <c r="B28" s="101"/>
+      <c r="C28" s="101"/>
+      <c r="D28" s="101"/>
       <c r="E28" s="33"/>
-      <c r="F28" s="148"/>
-      <c r="G28" s="148"/>
+      <c r="F28" s="102"/>
+      <c r="G28" s="102"/>
       <c r="H28" s="38"/>
       <c r="I28" s="39"/>
       <c r="J28" s="39"/>
@@ -2955,25 +2963,6 @@
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="BLIAlMBPgqH+NPEse4s68RjHq+iBp2ZxiPwbr85ja6anELCVKxbZV0o63eupwo+XV0ZheD91KVylaqjLC4V1wA==" saltValue="5R/Fmu0ewxRZ2Clu6FEY8g==" spinCount="100000" sheet="1" formatCells="0" formatColumns="0" formatRows="0"/>
   <mergeCells count="28">
-    <mergeCell ref="B18:F19"/>
-    <mergeCell ref="B20:D28"/>
-    <mergeCell ref="F24:G28"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="B13:F13"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="I16:L16"/>
-    <mergeCell ref="I17:L17"/>
-    <mergeCell ref="I21:J21"/>
-    <mergeCell ref="I22:J22"/>
-    <mergeCell ref="I23:J23"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="I15:L15"/>
-    <mergeCell ref="B4:F5"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="B9:C12"/>
-    <mergeCell ref="F6:F7"/>
     <mergeCell ref="M14:O14"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="M5:N5"/>
@@ -2983,6 +2972,25 @@
     <mergeCell ref="C3:E3"/>
     <mergeCell ref="L1:O3"/>
     <mergeCell ref="I14:L14"/>
+    <mergeCell ref="I15:L15"/>
+    <mergeCell ref="B4:F5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="B9:C12"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="I16:L16"/>
+    <mergeCell ref="I17:L17"/>
+    <mergeCell ref="I21:J21"/>
+    <mergeCell ref="I22:J22"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="B18:F19"/>
+    <mergeCell ref="B20:D28"/>
+    <mergeCell ref="F24:G28"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="G6:G7"/>
   </mergeCells>
   <conditionalFormatting sqref="B8:C8 F8:F12 H21:H23 E21:E28">
     <cfRule type="expression" dxfId="10" priority="1">
@@ -3116,6 +3124,168 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8125C971-851F-47D6-891B-0D146EC990A5}">
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="193">
+        <v>1</v>
+      </c>
+      <c r="F1" s="192" t="str">
+        <f ca="1">IF(M1="ACTIVE", "✓ Tracking Active", "⚠️ ERROR: Enable Iterative Calculations (File &gt; Options &gt; Formulas)")</f>
+        <v>✓ Tracking Active</v>
+      </c>
+      <c r="G1" s="192"/>
+      <c r="H1" s="192"/>
+      <c r="I1" s="192"/>
+      <c r="J1" s="192"/>
+      <c r="K1" s="192"/>
+      <c r="L1" s="192"/>
+      <c r="M1" s="1" t="str">
+        <f ca="1">IF(M1="ACTIVE", "ACTIVE", "ACTIVE")</f>
+        <v>ACTIVE</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A3,A3,A2)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A4,A4,A3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A5,A5,A4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A6,A6,A5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A7,A7,A6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A8,A8,A7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A9,A9,A8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A10,A10,A9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A11,A11,A10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A12,A12,A11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A13,A13,A12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A14,A14,A13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A15,A15,A14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A16,A16,A15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A17,A17,A16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A18,A18,A17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A19,A19,A18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A20,A20,A19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="str">
+        <f ca="1">IF('Basic Excel Formulas'!H$2&lt;&gt;A21,A21,A20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="str">
+        <f ca="1">IF(C$1="","",IF('Basic Excel Formulas'!H$2&lt;&gt;A21,'Basic Excel Formulas'!H$2,A21))</f>
+        <v>Your Name Here</v>
+      </c>
+    </row>
+  </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="buGetn6FOVTsLzeoKHutap1K9LElzOSIyBuEL+1QrE+hHN8SECVE9wIUOzGasnFCKh5ijjUSrXdMNwtlVIMJFw==" saltValue="fO1W8kXOsA43sZhUhgOW2g==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <mergeCells count="1">
+    <mergeCell ref="F1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE723ACA-9738-4B60-95AB-B3B2AD139FFF}">
   <dimension ref="B1:O25"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3133,13 +3303,13 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B2" s="166" t="s">
+      <c r="B2" s="158" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="167"/>
-      <c r="D2" s="167"/>
-      <c r="E2" s="167"/>
-      <c r="F2" s="168"/>
+      <c r="C2" s="159"/>
+      <c r="D2" s="159"/>
+      <c r="E2" s="159"/>
+      <c r="F2" s="160"/>
       <c r="L2" s="46">
         <v>1</v>
       </c>
@@ -3156,11 +3326,11 @@
       </c>
     </row>
     <row r="3" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="169"/>
-      <c r="C3" s="170"/>
-      <c r="D3" s="170"/>
-      <c r="E3" s="170"/>
-      <c r="F3" s="171"/>
+      <c r="B3" s="161"/>
+      <c r="C3" s="162"/>
+      <c r="D3" s="162"/>
+      <c r="E3" s="162"/>
+      <c r="F3" s="163"/>
       <c r="L3" s="46">
         <v>2</v>
       </c>
@@ -3172,17 +3342,17 @@
       </c>
     </row>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="175" t="s">
+      <c r="B4" s="164" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="176"/>
-      <c r="D4" s="177" t="s">
+      <c r="C4" s="165"/>
+      <c r="D4" s="166" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="179" t="s">
+      <c r="E4" s="168" t="s">
         <v>19</v>
       </c>
-      <c r="F4" s="181" t="s">
+      <c r="F4" s="170" t="s">
         <v>20</v>
       </c>
       <c r="G4" s="45"/>
@@ -3203,9 +3373,9 @@
       <c r="C5" s="50" t="s">
         <v>24</v>
       </c>
-      <c r="D5" s="178"/>
-      <c r="E5" s="180"/>
-      <c r="F5" s="182"/>
+      <c r="D5" s="167"/>
+      <c r="E5" s="169"/>
+      <c r="F5" s="171"/>
       <c r="L5" s="46">
         <v>4</v>
       </c>
@@ -3239,10 +3409,10 @@
       </c>
     </row>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="160" t="s">
+      <c r="B7" s="174" t="s">
         <v>74</v>
       </c>
-      <c r="C7" s="161"/>
+      <c r="C7" s="175"/>
       <c r="D7" s="51" t="s">
         <v>33</v>
       </c>
@@ -3263,8 +3433,8 @@
       </c>
     </row>
     <row r="8" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="162"/>
-      <c r="C8" s="163"/>
+      <c r="B8" s="176"/>
+      <c r="C8" s="177"/>
       <c r="D8" s="51" t="s">
         <v>38</v>
       </c>
@@ -3287,8 +3457,8 @@
       <c r="N8" s="48"/>
     </row>
     <row r="9" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="162"/>
-      <c r="C9" s="163"/>
+      <c r="B9" s="176"/>
+      <c r="C9" s="177"/>
       <c r="D9" s="51" t="s">
         <v>43</v>
       </c>
@@ -3313,8 +3483,8 @@
       <c r="N9" s="55"/>
     </row>
     <row r="10" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="164"/>
-      <c r="C10" s="165"/>
+      <c r="B10" s="178"/>
+      <c r="C10" s="179"/>
       <c r="D10" s="56" t="s">
         <v>48</v>
       </c>
@@ -3347,19 +3517,19 @@
     <row r="12" spans="2:15" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B12" s="59"/>
       <c r="I12" s="46"/>
-      <c r="M12" s="158" t="s">
+      <c r="M12" s="172" t="s">
         <v>75</v>
       </c>
-      <c r="N12" s="159"/>
+      <c r="N12" s="173"/>
     </row>
     <row r="13" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B13" s="166" t="s">
+      <c r="B13" s="158" t="s">
         <v>59</v>
       </c>
-      <c r="C13" s="167"/>
-      <c r="D13" s="167"/>
-      <c r="E13" s="167"/>
-      <c r="F13" s="168"/>
+      <c r="C13" s="159"/>
+      <c r="D13" s="159"/>
+      <c r="E13" s="159"/>
+      <c r="F13" s="160"/>
       <c r="M13" s="60" t="s">
         <v>25</v>
       </c>
@@ -3368,11 +3538,11 @@
       </c>
     </row>
     <row r="14" spans="2:15" ht="17.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="169"/>
-      <c r="C14" s="170"/>
-      <c r="D14" s="170"/>
-      <c r="E14" s="170"/>
-      <c r="F14" s="171"/>
+      <c r="B14" s="161"/>
+      <c r="C14" s="162"/>
+      <c r="D14" s="162"/>
+      <c r="E14" s="162"/>
+      <c r="F14" s="163"/>
       <c r="M14" s="60" t="s">
         <v>30</v>
       </c>
@@ -3381,11 +3551,11 @@
       </c>
     </row>
     <row r="15" spans="2:15" ht="17.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="172" t="s">
+      <c r="B15" s="180" t="s">
         <v>76</v>
       </c>
-      <c r="C15" s="172"/>
-      <c r="D15" s="172"/>
+      <c r="C15" s="180"/>
+      <c r="D15" s="180"/>
       <c r="E15" s="62" t="s">
         <v>60</v>
       </c>
@@ -3406,9 +3576,9 @@
       </c>
     </row>
     <row r="16" spans="2:15" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="173"/>
-      <c r="C16" s="173"/>
-      <c r="D16" s="173"/>
+      <c r="B16" s="181"/>
+      <c r="C16" s="181"/>
+      <c r="D16" s="181"/>
       <c r="E16" s="66"/>
       <c r="F16" s="51" t="s">
         <v>64</v>
@@ -3432,9 +3602,9 @@
       </c>
     </row>
     <row r="17" spans="2:14" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="173"/>
-      <c r="C17" s="173"/>
-      <c r="D17" s="173"/>
+      <c r="B17" s="181"/>
+      <c r="C17" s="181"/>
+      <c r="D17" s="181"/>
       <c r="E17" s="66"/>
       <c r="F17" s="51" t="s">
         <v>67</v>
@@ -3458,9 +3628,9 @@
       </c>
     </row>
     <row r="18" spans="2:14" ht="14.45" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="173"/>
-      <c r="C18" s="173"/>
-      <c r="D18" s="173"/>
+      <c r="B18" s="181"/>
+      <c r="C18" s="181"/>
+      <c r="D18" s="181"/>
       <c r="E18" s="66"/>
       <c r="F18" s="51" t="s">
         <v>70</v>
@@ -3478,68 +3648,68 @@
       </c>
     </row>
     <row r="19" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B19" s="173"/>
-      <c r="C19" s="173"/>
-      <c r="D19" s="173"/>
+      <c r="B19" s="181"/>
+      <c r="C19" s="181"/>
+      <c r="D19" s="181"/>
       <c r="E19" s="66"/>
-      <c r="F19" s="174" t="s">
+      <c r="F19" s="182" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="174"/>
+      <c r="G19" s="182"/>
     </row>
     <row r="20" spans="2:14" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="173"/>
-      <c r="C20" s="173"/>
-      <c r="D20" s="173"/>
+      <c r="B20" s="181"/>
+      <c r="C20" s="181"/>
+      <c r="D20" s="181"/>
       <c r="E20" s="66"/>
-      <c r="F20" s="174"/>
-      <c r="G20" s="174"/>
+      <c r="F20" s="182"/>
+      <c r="G20" s="182"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B21" s="173"/>
-      <c r="C21" s="173"/>
-      <c r="D21" s="173"/>
+      <c r="B21" s="181"/>
+      <c r="C21" s="181"/>
+      <c r="D21" s="181"/>
       <c r="E21" s="66"/>
-      <c r="F21" s="174"/>
-      <c r="G21" s="174"/>
+      <c r="F21" s="182"/>
+      <c r="G21" s="182"/>
     </row>
     <row r="22" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B22" s="173"/>
-      <c r="C22" s="173"/>
-      <c r="D22" s="173"/>
+      <c r="B22" s="181"/>
+      <c r="C22" s="181"/>
+      <c r="D22" s="181"/>
       <c r="E22" s="66"/>
-      <c r="F22" s="174"/>
-      <c r="G22" s="174"/>
+      <c r="F22" s="182"/>
+      <c r="G22" s="182"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B23" s="173"/>
-      <c r="C23" s="173"/>
-      <c r="D23" s="173"/>
+      <c r="B23" s="181"/>
+      <c r="C23" s="181"/>
+      <c r="D23" s="181"/>
       <c r="E23" s="66"/>
-      <c r="F23" s="174"/>
-      <c r="G23" s="174"/>
+      <c r="F23" s="182"/>
+      <c r="G23" s="182"/>
     </row>
     <row r="25" spans="2:14" ht="17.45" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="OpD0C6psjTe/kStoo1h7yvA+15jkxfWm/NBH5QdNDZMthMHZ8e+D8fccabo00cUHiBPBG012UpwlWS/LhPlnkg==" saltValue="T+6KfbnqR49JhNBhr/3oaA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="10">
+    <mergeCell ref="M12:N12"/>
+    <mergeCell ref="B7:C10"/>
+    <mergeCell ref="B13:F14"/>
+    <mergeCell ref="B15:D23"/>
+    <mergeCell ref="F19:G23"/>
     <mergeCell ref="B2:F3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="F4:F5"/>
-    <mergeCell ref="M12:N12"/>
-    <mergeCell ref="B7:C10"/>
-    <mergeCell ref="B13:F14"/>
-    <mergeCell ref="B15:D23"/>
-    <mergeCell ref="F19:G23"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{262A2B2D-0544-4AF4-8F48-1115B33F73A4}">
   <dimension ref="B1:F5"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3587,6 +3757,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cca9fd2d-ef84-45c9-8063-8f4bd4c29606">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002C289946819CFF499E91D197BC975371" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="674b7a4e239a9748c7aaa97e309327a4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cca9fd2d-ef84-45c9-8063-8f4bd4c29606" xmlns:ns3="18557d39-01b8-4d71-9479-3fad465290ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="600253478e594d1349e02792803dc53a" ns2:_="" ns3:_="">
     <xsd:import namespace="cca9fd2d-ef84-45c9-8063-8f4bd4c29606"/>
@@ -3803,26 +3992,25 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4FB4873-1F2B-4DA5-A59D-EA2845F46BB6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cca9fd2d-ef84-45c9-8063-8f4bd4c29606"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cca9fd2d-ef84-45c9-8063-8f4bd4c29606">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42C52D6A-E0AB-44E7-ABE4-D928B05D246F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A2CE780C-3974-4A71-8F18-23A7FE356660}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3839,22 +4027,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42C52D6A-E0AB-44E7-ABE4-D928B05D246F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4FB4873-1F2B-4DA5-A59D-EA2845F46BB6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="cca9fd2d-ef84-45c9-8063-8f4bd4c29606"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>